<commit_message>
correcting pH data for ID 35 adn 58
</commit_message>
<xml_diff>
--- a/reductions-lit/data/lit_dat.xlsx
+++ b/reductions-lit/data/lit_dat.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://aarhusuniversitet-my.sharepoint.com/personal/au583430_uni_au_dk/Documents/Documents/GitHub/GD-NH3/reductions/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://aarhusuniversitet-my.sharepoint.com/personal/au583430_uni_au_dk/Documents/Documents/GitHub/GD-NH3/reductions-lit/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="219" documentId="8_{7C4171F8-D199-4843-B714-C3F258BC4D93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D484913B-73F5-43B3-A6A4-9D9DF7B62CB7}"/>
+  <xr:revisionPtr revIDLastSave="233" documentId="8_{7C4171F8-D199-4843-B714-C3F258BC4D93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{40461209-7FEB-4794-8967-57D2A0E2342A}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{DF353E34-80BC-440D-84E6-1A1BEACE8767}"/>
   </bookViews>
@@ -4828,7 +4828,8 @@
     <col min="22" max="22" width="7.5703125" style="1" customWidth="1"/>
     <col min="23" max="23" width="9.140625" style="2" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="10.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="25" max="26" width="10.5703125" style="2" customWidth="1"/>
+    <col min="25" max="25" width="19.140625" style="2" customWidth="1"/>
+    <col min="26" max="26" width="10.5703125" style="2" customWidth="1"/>
     <col min="27" max="28" width="9.42578125" style="2" customWidth="1"/>
     <col min="29" max="29" width="20.42578125" style="2" customWidth="1"/>
     <col min="30" max="31" width="44.5703125" style="1" customWidth="1"/>
@@ -23993,7 +23994,7 @@
         <v>0.17</v>
       </c>
       <c r="V137" s="1">
-        <v>6.4</v>
+        <v>6.5</v>
       </c>
       <c r="W137" s="2">
         <v>35</v>
@@ -24134,7 +24135,7 @@
         <v>0.1</v>
       </c>
       <c r="V138" s="1">
-        <v>5.9</v>
+        <v>6.5</v>
       </c>
       <c r="W138" s="2">
         <v>35</v>
@@ -24275,7 +24276,7 @@
         <v>0.2</v>
       </c>
       <c r="V139" s="1">
-        <v>6.4</v>
+        <v>7</v>
       </c>
       <c r="W139" s="2">
         <v>35</v>
@@ -24416,7 +24417,7 @@
         <v>0.15</v>
       </c>
       <c r="V140" s="1">
-        <v>5.9</v>
+        <v>7</v>
       </c>
       <c r="W140" s="2">
         <v>35</v>
@@ -24557,7 +24558,7 @@
         <v>0.03</v>
       </c>
       <c r="V141" s="1">
-        <v>6.5</v>
+        <v>7</v>
       </c>
       <c r="W141" s="2">
         <v>35</v>
@@ -24698,7 +24699,7 @@
         <v>0.03</v>
       </c>
       <c r="V142" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="W142" s="2">
         <v>35</v>
@@ -24839,7 +24840,7 @@
         <v>0.13</v>
       </c>
       <c r="V143" s="1">
-        <v>6.3</v>
+        <v>6.9</v>
       </c>
       <c r="W143" s="2">
         <v>35</v>
@@ -24980,7 +24981,7 @@
         <v>0.03</v>
       </c>
       <c r="V144" s="8">
-        <v>6.1</v>
+        <v>6.9</v>
       </c>
       <c r="W144" s="11">
         <v>35</v>
@@ -44482,7 +44483,7 @@
       <c r="T281" s="1"/>
       <c r="U281" s="1"/>
       <c r="V281" s="1">
-        <v>5.6</v>
+        <v>7.2</v>
       </c>
       <c r="X281" s="2">
         <v>84.8</v>
@@ -44697,7 +44698,7 @@
       <c r="T283"/>
       <c r="U283"/>
       <c r="V283" s="1">
-        <v>5.7</v>
+        <v>7.5</v>
       </c>
       <c r="W283"/>
       <c r="X283" s="2">

</xml_diff>